<commit_message>
docs: update copyright year and fix various documentation issues
- Update copyright year from 2025 to 2026 in _config.yml
- Fix citation references in congestion.ipynb
- Add FontAwesome license file
- Adjust sidebar width in CSS
- Update Jupyter notebook metadata and execution counts
- Add error log file for failed notebook execution
- Improve toggle button accessibility and functionality
- Update search index and static assets
</commit_message>
<xml_diff>
--- a/_build/html/_downloads/f5cac977ce6872d68fcaf5cd7a8258b4/congestion_indices.xlsx
+++ b/_build/html/_downloads/f5cac977ce6872d68fcaf5cd7a8258b4/congestion_indices.xlsx
@@ -1,21 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24334"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yiliangli/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Zhongjun\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{548A798E-E56B-6D4A-BB0A-6D7DB95BD221}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE865978-23B2-4B55-9E87-C919DF6B02FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34560" windowHeight="20120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="18746" yWindow="2014" windowWidth="22671" windowHeight="15772" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="124519"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -35,10 +40,24 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="177" formatCode="#,##0.000;[Red]\-#,##0.000"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
-      <name val="Calibri"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -49,21 +68,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -77,14 +82,28 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <dxfs count="3">
+    <dxf>
+      <numFmt numFmtId="177" formatCode="#,##0.000;[Red]\-#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="177" formatCode="#,##0.000;[Red]\-#,##0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd;@"/>
+    </dxf>
+  </dxfs>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -96,8 +115,20 @@
 </styleSheet>
 </file>
 
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Frame0" displayName="Frame0" ref="A1:C124" totalsRowShown="0">
+  <autoFilter ref="A1:C124" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="date" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="ACT" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="ACR" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 主题​​">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -107,44 +138,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -191,12 +222,12 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -252,171 +283,178 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
-            <a:schemeClr val="phClr"/>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C112"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:C124"/>
+  <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.3046875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -427,7 +465,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>42370</v>
       </c>
@@ -435,10 +473,10 @@
         <v>6.7340446561307958</v>
       </c>
       <c r="C2" s="2">
-        <v>32.501772230295316</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+        <v>32.501772230295323</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>42401</v>
       </c>
@@ -449,7 +487,7 @@
         <v>30.52942593037589</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>42430</v>
       </c>
@@ -457,10 +495,10 @@
         <v>6.3517051756594878</v>
       </c>
       <c r="C4" s="2">
-        <v>31.163417830133653</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+        <v>31.16341783013365</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>42461</v>
       </c>
@@ -471,7 +509,7 @@
         <v>34.099178540987893</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>42491</v>
       </c>
@@ -482,7 +520,7 @@
         <v>32.384593319774822</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>42522</v>
       </c>
@@ -490,10 +528,10 @@
         <v>5.9991617331631248</v>
       </c>
       <c r="C7" s="2">
-        <v>31.478672227662678</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+        <v>31.478672227662681</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>42552</v>
       </c>
@@ -501,21 +539,21 @@
         <v>5.6322038179292591</v>
       </c>
       <c r="C8" s="2">
-        <v>31.155919956222203</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+        <v>31.155919956222199</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>42583</v>
       </c>
       <c r="B9" s="2">
-        <v>5.3063771569587495</v>
+        <v>5.3063771569587486</v>
       </c>
       <c r="C9" s="2">
         <v>30.260259274678809</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>42614</v>
       </c>
@@ -523,10 +561,10 @@
         <v>4.8844875556454159</v>
       </c>
       <c r="C10" s="2">
-        <v>29.462751037879922</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+        <v>29.462751037879919</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>42644</v>
       </c>
@@ -534,10 +572,10 @@
         <v>5.4723077717028277</v>
       </c>
       <c r="C11" s="2">
-        <v>29.911096126967806</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+        <v>29.911096126967809</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>42675</v>
       </c>
@@ -545,10 +583,10 @@
         <v>5.5055288164874696</v>
       </c>
       <c r="C12" s="2">
-        <v>31.561280805827618</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+        <v>31.561280805827622</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>42705</v>
       </c>
@@ -559,7 +597,7 @@
         <v>30.736966680320329</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>42736</v>
       </c>
@@ -567,10 +605,10 @@
         <v>6.9821139181318239</v>
       </c>
       <c r="C14" s="2">
-        <v>31.837631331576635</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+        <v>31.837631331576631</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>42767</v>
       </c>
@@ -578,10 +616,10 @@
         <v>5.4137889421406209</v>
       </c>
       <c r="C15" s="2">
-        <v>28.945512810879723</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+        <v>28.94551281087972</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>42795</v>
       </c>
@@ -589,10 +627,10 @@
         <v>5.5999738442135714</v>
       </c>
       <c r="C16" s="2">
-        <v>29.701869378523075</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+        <v>29.701869378523071</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>42826</v>
       </c>
@@ -600,10 +638,10 @@
         <v>6.8222869257472762</v>
       </c>
       <c r="C17" s="2">
-        <v>32.370188679775374</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+        <v>32.370188679775367</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>42856</v>
       </c>
@@ -611,10 +649,10 @@
         <v>6.2337282321643057</v>
       </c>
       <c r="C18" s="2">
-        <v>31.480007400831767</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+        <v>31.48000740083177</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>42887</v>
       </c>
@@ -622,10 +660,10 @@
         <v>5.3295612314756138</v>
       </c>
       <c r="C19" s="2">
-        <v>29.470505675109553</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+        <v>29.47050567510955</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>42917</v>
       </c>
@@ -636,7 +674,7 @@
         <v>28.904546240002151</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>42948</v>
       </c>
@@ -644,10 +682,10 @@
         <v>5.2527974034305416</v>
       </c>
       <c r="C21" s="2">
-        <v>29.190156030416542</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+        <v>29.190156030416539</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>42979</v>
       </c>
@@ -655,10 +693,10 @@
         <v>4.623108365912775</v>
       </c>
       <c r="C22" s="2">
-        <v>27.725331260347875</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+        <v>27.725331260347879</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>43009</v>
       </c>
@@ -666,10 +704,10 @@
         <v>5.024929266679214</v>
       </c>
       <c r="C23" s="2">
-        <v>27.344328650472374</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+        <v>27.34432865047237</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>43040</v>
       </c>
@@ -677,10 +715,10 @@
         <v>5.285800859191168</v>
       </c>
       <c r="C24" s="2">
-        <v>26.864592038576696</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+        <v>26.864592038576699</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>43070</v>
       </c>
@@ -688,10 +726,10 @@
         <v>5.1690420939105888</v>
       </c>
       <c r="C25" s="2">
-        <v>27.701826942726854</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+        <v>27.70182694272685</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>43101</v>
       </c>
@@ -699,10 +737,10 @@
         <v>5.9920525957915807</v>
       </c>
       <c r="C26" s="2">
-        <v>27.740110334655014</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+        <v>27.740110334655011</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>43132</v>
       </c>
@@ -710,10 +748,10 @@
         <v>6.1950208729644212</v>
       </c>
       <c r="C27" s="2">
-        <v>27.255426916942007</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+        <v>27.25542691694201</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>43160</v>
       </c>
@@ -721,21 +759,21 @@
         <v>6.3990291136274191</v>
       </c>
       <c r="C28" s="2">
-        <v>28.447872682324387</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+        <v>28.447872682324391</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>43191</v>
       </c>
       <c r="B29" s="2">
-        <v>6.3110442003427725</v>
+        <v>6.3110442003427716</v>
       </c>
       <c r="C29" s="2">
-        <v>29.166034648146574</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+        <v>29.166034648146571</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>43221</v>
       </c>
@@ -746,7 +784,7 @@
         <v>29.660451394803911</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>43252</v>
       </c>
@@ -757,7 +795,7 @@
         <v>28.125243004822529</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>43282</v>
       </c>
@@ -765,10 +803,10 @@
         <v>5.949829833397744</v>
       </c>
       <c r="C32" s="2">
-        <v>28.048600338468436</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+        <v>28.048600338468439</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
         <v>43313</v>
       </c>
@@ -776,10 +814,10 @@
         <v>6.662998299711993</v>
       </c>
       <c r="C33" s="2">
-        <v>29.238868295738257</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+        <v>29.238868295738261</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
         <v>43344</v>
       </c>
@@ -790,40 +828,40 @@
         <v>28.183721026928769</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
         <v>43374</v>
       </c>
       <c r="B35" s="2">
-        <v>5.6823046735758584</v>
+        <v>5.6823046735758576</v>
       </c>
       <c r="C35" s="2">
-        <v>27.222558982500434</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+        <v>27.222558982500431</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
         <v>43405</v>
       </c>
       <c r="B36" s="2">
-        <v>5.6992339009120645</v>
+        <v>5.6992339009120636</v>
       </c>
       <c r="C36" s="2">
-        <v>28.035544521988363</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+        <v>28.03554452198836</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" s="1">
         <v>43435</v>
       </c>
       <c r="B37" s="2">
-        <v>5.3364798992614855</v>
+        <v>5.3364798992614846</v>
       </c>
       <c r="C37" s="2">
-        <v>27.000415982085386</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+        <v>27.000415982085389</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" s="1">
         <v>43466</v>
       </c>
@@ -834,7 +872,7 @@
         <v>26.159118485660429</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" s="1">
         <v>43497</v>
       </c>
@@ -842,10 +880,10 @@
         <v>5.6650140059851228</v>
       </c>
       <c r="C39" s="2">
-        <v>25.502893039008683</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+        <v>25.502893039008679</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" s="1">
         <v>43525</v>
       </c>
@@ -853,10 +891,10 @@
         <v>5.298851133192211</v>
       </c>
       <c r="C40" s="2">
-        <v>26.649029813354996</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+        <v>26.649029813355</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" s="1">
         <v>43556</v>
       </c>
@@ -867,7 +905,7 @@
         <v>28.809173162482519</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" s="1">
         <v>43586</v>
       </c>
@@ -878,7 +916,7 @@
         <v>28.585457910946079</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" s="1">
         <v>43617</v>
       </c>
@@ -889,7 +927,7 @@
         <v>26.68718764087744</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" s="1">
         <v>43647</v>
       </c>
@@ -897,10 +935,10 @@
         <v>4.9454755865762596</v>
       </c>
       <c r="C44" s="2">
-        <v>25.593433079129294</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+        <v>25.593433079129291</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" s="1">
         <v>43678</v>
       </c>
@@ -908,10 +946,10 @@
         <v>5.2129584393609933</v>
       </c>
       <c r="C45" s="2">
-        <v>26.924884562533258</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+        <v>26.924884562533261</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" s="1">
         <v>43709</v>
       </c>
@@ -919,10 +957,10 @@
         <v>4.8047806158569752</v>
       </c>
       <c r="C46" s="2">
-        <v>25.990418682866796</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+        <v>25.9904186828668</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" s="1">
         <v>43739</v>
       </c>
@@ -933,7 +971,7 @@
         <v>25.144376648804791</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" s="1">
         <v>43770</v>
       </c>
@@ -944,7 +982,7 @@
         <v>25.218789546596039</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" s="1">
         <v>43800</v>
       </c>
@@ -952,10 +990,10 @@
         <v>4.9055952700909797</v>
       </c>
       <c r="C49" s="2">
-        <v>25.578284062076456</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+        <v>25.57828406207646</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" s="1">
         <v>43831</v>
       </c>
@@ -963,10 +1001,10 @@
         <v>5.7141785867858834</v>
       </c>
       <c r="C50" s="2">
-        <v>25.979345870821955</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+        <v>25.979345870821959</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A51" s="1">
         <v>43862</v>
       </c>
@@ -974,21 +1012,21 @@
         <v>5.4084815515862763</v>
       </c>
       <c r="C51" s="2">
-        <v>25.165326573888436</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+        <v>25.165326573888439</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" s="1">
         <v>43891</v>
       </c>
       <c r="B52" s="2">
-        <v>5.5573089689030555</v>
+        <v>5.5573089689030546</v>
       </c>
       <c r="C52" s="2">
-        <v>27.458445917167545</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+        <v>27.458445917167541</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" s="1">
         <v>43922</v>
       </c>
@@ -996,10 +1034,10 @@
         <v>5.625923230454684</v>
       </c>
       <c r="C53" s="2">
-        <v>26.013312660213213</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+        <v>26.013312660213209</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" s="1">
         <v>43952</v>
       </c>
@@ -1010,7 +1048,7 @@
         <v>27.103771708600679</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" s="1">
         <v>43983</v>
       </c>
@@ -1018,10 +1056,10 @@
         <v>5.5107770041913433</v>
       </c>
       <c r="C55" s="2">
-        <v>27.392504201407412</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+        <v>27.392504201407409</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" s="1">
         <v>44013</v>
       </c>
@@ -1029,10 +1067,10 @@
         <v>5.3208206212709266</v>
       </c>
       <c r="C56" s="2">
-        <v>26.574783739867485</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+        <v>26.574783739867481</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" s="1">
         <v>44044</v>
       </c>
@@ -1040,10 +1078,10 @@
         <v>5.9558249198004871</v>
       </c>
       <c r="C57" s="2">
-        <v>28.498393253916106</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+        <v>28.49839325391611</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58" s="1">
         <v>44075</v>
       </c>
@@ -1054,7 +1092,7 @@
         <v>28.903288204070101</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59" s="1">
         <v>44105</v>
       </c>
@@ -1062,10 +1100,10 @@
         <v>6.109573059916233</v>
       </c>
       <c r="C59" s="2">
-        <v>28.228192711896185</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+        <v>28.228192711896181</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60" s="1">
         <v>44136</v>
       </c>
@@ -1073,10 +1111,10 @@
         <v>7.2125656733969024</v>
       </c>
       <c r="C60" s="2">
-        <v>29.366151390515146</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+        <v>29.366151390515149</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61" s="1">
         <v>44166</v>
       </c>
@@ -1087,18 +1125,18 @@
         <v>28.98522643550276</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A62" s="1">
         <v>44197</v>
       </c>
       <c r="B62" s="2">
-        <v>10.770924993688775</v>
+        <v>10.770924993688769</v>
       </c>
       <c r="C62" s="2">
-        <v>34.364240507426786</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+        <v>34.364240507426793</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63" s="1">
         <v>44228</v>
       </c>
@@ -1109,7 +1147,7 @@
         <v>33.099751646972393</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A64" s="1">
         <v>44256</v>
       </c>
@@ -1120,7 +1158,7 @@
         <v>33.637338836392239</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" s="1">
         <v>44287</v>
       </c>
@@ -1128,10 +1166,10 @@
         <v>8.9902566668822033</v>
       </c>
       <c r="C65" s="2">
-        <v>34.366088154992916</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+        <v>34.366088154992923</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" s="1">
         <v>44317</v>
       </c>
@@ -1142,29 +1180,29 @@
         <v>36.378162597166273</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" s="1">
         <v>44348</v>
       </c>
       <c r="B67" s="2">
-        <v>12.803494259241015</v>
+        <v>12.80349425924102</v>
       </c>
       <c r="C67" s="2">
         <v>38.212874832438423</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68" s="1">
         <v>44378</v>
       </c>
       <c r="B68" s="2">
-        <v>12.248897070224114</v>
+        <v>12.24889707022411</v>
       </c>
       <c r="C68" s="2">
-        <v>36.819292745113984</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+        <v>36.819292745113977</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" s="1">
         <v>44409</v>
       </c>
@@ -1175,7 +1213,7 @@
         <v>35.576575761735839</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70" s="1">
         <v>44440</v>
       </c>
@@ -1186,29 +1224,29 @@
         <v>37.182770248999319</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71" s="1">
         <v>44470</v>
       </c>
       <c r="B71" s="2">
-        <v>12.956912783153282</v>
+        <v>12.95691278315328</v>
       </c>
       <c r="C71" s="2">
         <v>35.442007116689169</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A72" s="1">
         <v>44501</v>
       </c>
       <c r="B72" s="2">
-        <v>11.266483849410811</v>
+        <v>11.266483849410809</v>
       </c>
       <c r="C72" s="2">
         <v>35.391166775975819</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A73" s="1">
         <v>44531</v>
       </c>
@@ -1219,18 +1257,18 @@
         <v>33.851465263584629</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A74" s="1">
         <v>44562</v>
       </c>
       <c r="B74" s="2">
-        <v>10.268272263306798</v>
+        <v>10.2682722633068</v>
       </c>
       <c r="C74" s="2">
         <v>34.966510103445003</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A75" s="1">
         <v>44593</v>
       </c>
@@ -1238,65 +1276,65 @@
         <v>8.211507997929921</v>
       </c>
       <c r="C75" s="2">
-        <v>32.641133365099435</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
+        <v>32.641133365099442</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A76" s="1">
         <v>44621</v>
       </c>
       <c r="B76" s="2">
-        <v>10.641169104631599</v>
+        <v>10.641169104631601</v>
       </c>
       <c r="C76" s="2">
         <v>35.189421580935843</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A77" s="1">
         <v>44652</v>
       </c>
       <c r="B77" s="2">
-        <v>11.362650966603779</v>
+        <v>11.36265096660378</v>
       </c>
       <c r="C77" s="2">
         <v>37.477118893119609</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A78" s="1">
         <v>44682</v>
       </c>
       <c r="B78" s="2">
-        <v>12.121543724511284</v>
+        <v>12.12154372451128</v>
       </c>
       <c r="C78" s="2">
         <v>37.111541648332746</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A79" s="1">
         <v>44713</v>
       </c>
       <c r="B79" s="2">
-        <v>12.538175034813065</v>
+        <v>12.53817503481307</v>
       </c>
       <c r="C79" s="2">
-        <v>36.921837080864705</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
+        <v>36.921837080864712</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A80" s="1">
         <v>44743</v>
       </c>
       <c r="B80" s="2">
-        <v>11.219226332259597</v>
+        <v>11.2192263322596</v>
       </c>
       <c r="C80" s="2">
-        <v>36.441305561010154</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
+        <v>36.441305561010147</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A81" s="1">
         <v>44774</v>
       </c>
@@ -1304,10 +1342,10 @@
         <v>9.7637122078254883</v>
       </c>
       <c r="C81" s="2">
-        <v>33.958546089070175</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
+        <v>33.958546089070182</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A82" s="1">
         <v>44805</v>
       </c>
@@ -1315,10 +1353,10 @@
         <v>9.0378919986691582</v>
       </c>
       <c r="C82" s="2">
-        <v>33.055274195868975</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
+        <v>33.055274195868982</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A83" s="1">
         <v>44835</v>
       </c>
@@ -1329,7 +1367,7 @@
         <v>32.449506591589241</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A84" s="1">
         <v>44866</v>
       </c>
@@ -1337,10 +1375,10 @@
         <v>8.754484169433411</v>
       </c>
       <c r="C84" s="2">
-        <v>33.148027750967344</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
+        <v>33.148027750967337</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A85" s="1">
         <v>44896</v>
       </c>
@@ -1351,7 +1389,7 @@
         <v>31.75674002829658</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A86" s="1">
         <v>44927</v>
       </c>
@@ -1359,10 +1397,10 @@
         <v>8.8708633177229608</v>
       </c>
       <c r="C86" s="2">
-        <v>31.363168168545084</v>
-      </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
+        <v>31.36316816854508</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A87" s="1">
         <v>44958</v>
       </c>
@@ -1373,7 +1411,7 @@
         <v>29.32270530453944</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A88" s="1">
         <v>44986</v>
       </c>
@@ -1381,10 +1419,10 @@
         <v>7.3666389529473806</v>
       </c>
       <c r="C88" s="2">
-        <v>31.987864947444148</v>
-      </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
+        <v>31.987864947444152</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A89" s="1">
         <v>45017</v>
       </c>
@@ -1395,7 +1433,7 @@
         <v>33.317801620348618</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A90" s="1">
         <v>45047</v>
       </c>
@@ -1406,7 +1444,7 @@
         <v>31.39135148187232</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A91" s="1">
         <v>45078</v>
       </c>
@@ -1414,10 +1452,10 @@
         <v>7.1575268675491346</v>
       </c>
       <c r="C91" s="2">
-        <v>30.801694859331924</v>
-      </c>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
+        <v>30.801694859331921</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A92" s="1">
         <v>45108</v>
       </c>
@@ -1428,7 +1466,7 @@
         <v>29.1167356381325</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A93" s="1">
         <v>45139</v>
       </c>
@@ -1436,10 +1474,10 @@
         <v>6.6316803529969981</v>
       </c>
       <c r="C93" s="2">
-        <v>29.120719364931546</v>
-      </c>
-    </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
+        <v>29.120719364931549</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A94" s="1">
         <v>45170</v>
       </c>
@@ -1447,10 +1485,10 @@
         <v>6.5706655527947557</v>
       </c>
       <c r="C94" s="2">
-        <v>29.787720343289557</v>
-      </c>
-    </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
+        <v>29.787720343289561</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A95" s="1">
         <v>45200</v>
       </c>
@@ -1461,7 +1499,7 @@
         <v>27.729563786676849</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A96" s="1">
         <v>45231</v>
       </c>
@@ -1469,21 +1507,21 @@
         <v>6.6960367893902699</v>
       </c>
       <c r="C96" s="2">
-        <v>29.043098491692337</v>
-      </c>
-    </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
+        <v>29.043098491692341</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A97" s="1">
         <v>45261</v>
       </c>
       <c r="B97" s="2">
-        <v>7.1809551173220045</v>
+        <v>7.1809551173220054</v>
       </c>
       <c r="C97" s="2">
         <v>30.190208594941449</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A98" s="1">
         <v>45292</v>
       </c>
@@ -1491,10 +1529,10 @@
         <v>6.7556443616760307</v>
       </c>
       <c r="C98" s="2">
-        <v>28.706104270274636</v>
-      </c>
-    </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
+        <v>28.70610427027464</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A99" s="1">
         <v>45323</v>
       </c>
@@ -1502,10 +1540,10 @@
         <v>6.7219832498708874</v>
       </c>
       <c r="C99" s="2">
-        <v>27.029441036845366</v>
-      </c>
-    </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
+        <v>27.02944103684537</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A100" s="1">
         <v>45352</v>
       </c>
@@ -1516,7 +1554,7 @@
         <v>30.309078786230689</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A101" s="1">
         <v>45383</v>
       </c>
@@ -1527,7 +1565,7 @@
         <v>32.63871038704432</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A102" s="1">
         <v>45413</v>
       </c>
@@ -1535,10 +1573,10 @@
         <v>8.8663252021550178</v>
       </c>
       <c r="C102" s="2">
-        <v>31.811735211649488</v>
-      </c>
-    </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
+        <v>31.811735211649491</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A103" s="1">
         <v>45444</v>
       </c>
@@ -1549,7 +1587,7 @@
         <v>33.134973123269681</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A104" s="1">
         <v>45474</v>
       </c>
@@ -1560,7 +1598,7 @@
         <v>31.526135314898411</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A105" s="1">
         <v>45505</v>
       </c>
@@ -1568,10 +1606,10 @@
         <v>8.4005818410123023</v>
       </c>
       <c r="C105" s="2">
-        <v>30.709135101041444</v>
-      </c>
-    </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
+        <v>30.70913510104144</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A106" s="1">
         <v>45536</v>
       </c>
@@ -1579,10 +1617,10 @@
         <v>8.5669557410654846</v>
       </c>
       <c r="C106" s="2">
-        <v>30.780278899889684</v>
-      </c>
-    </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.2">
+        <v>30.78027889988968</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A107" s="1">
         <v>45566</v>
       </c>
@@ -1590,10 +1628,10 @@
         <v>8.6919412186209701</v>
       </c>
       <c r="C107" s="2">
-        <v>30.868938779126296</v>
-      </c>
-    </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.2">
+        <v>30.868938779126299</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A108" s="1">
         <v>45597</v>
       </c>
@@ -1604,7 +1642,7 @@
         <v>29.88793508659036</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A109" s="1">
         <v>45627</v>
       </c>
@@ -1615,7 +1653,7 @@
         <v>30.47315800005833</v>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A110" s="1">
         <v>45658</v>
       </c>
@@ -1626,7 +1664,7 @@
         <v>29.315217304939271</v>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A111" s="1">
         <v>45689</v>
       </c>
@@ -1637,7 +1675,7 @@
         <v>23.622837654290421</v>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A112" s="1">
         <v>45717</v>
       </c>
@@ -1645,10 +1683,147 @@
         <v>5.9318545537918759</v>
       </c>
       <c r="C112" s="2">
-        <v>24.785357796236088</v>
+        <v>24.785357796236092</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A113" s="1">
+        <v>45748</v>
+      </c>
+      <c r="B113" s="2">
+        <v>6.1263084342797454</v>
+      </c>
+      <c r="C113" s="2">
+        <v>25.79387825289465</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A114" s="1">
+        <v>45778</v>
+      </c>
+      <c r="B114" s="2">
+        <v>6.2789088614419448</v>
+      </c>
+      <c r="C114" s="2">
+        <v>25.964931627701809</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A115" s="1">
+        <v>45809</v>
+      </c>
+      <c r="B115" s="2">
+        <v>5.2855972464611209</v>
+      </c>
+      <c r="C115" s="2">
+        <v>24.41592073411023</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A116" s="1">
+        <v>45839</v>
+      </c>
+      <c r="B116" s="2">
+        <v>5.7825086891757698</v>
+      </c>
+      <c r="C116" s="2">
+        <v>23.85523557320975</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A117" s="1">
+        <v>45870</v>
+      </c>
+      <c r="B117" s="2">
+        <v>6.2280904944715507</v>
+      </c>
+      <c r="C117" s="2">
+        <v>24.91206172699421</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A118" s="1">
+        <v>45901</v>
+      </c>
+      <c r="B118" s="2">
+        <v>7.1678336762688613</v>
+      </c>
+      <c r="C118" s="2">
+        <v>24.403292181069961</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A119" s="1">
+        <v>45931</v>
+      </c>
+      <c r="B119" s="2">
+        <v>6.2793012209005612</v>
+      </c>
+      <c r="C119" s="2">
+        <v>23.29525379813921</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A120" s="1">
+        <v>45962</v>
+      </c>
+      <c r="B120" s="2">
+        <v>4.75918877801716</v>
+      </c>
+      <c r="C120" s="2">
+        <v>20.574895112824581</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A121" s="1">
+        <v>45992</v>
+      </c>
+      <c r="B121" s="2">
+        <v>3.9858272010712441</v>
+      </c>
+      <c r="C121" s="2">
+        <v>19.7096685839496</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A122" s="1">
+        <v>46023</v>
+      </c>
+      <c r="B122" s="2">
+        <v>5.1122706947032208</v>
+      </c>
+      <c r="C122" s="2">
+        <v>20.841096619643331</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A123" s="1">
+        <v>46054</v>
+      </c>
+      <c r="B123" s="2">
+        <v>6.1786166205253226</v>
+      </c>
+      <c r="C123" s="2">
+        <v>21.699516548902938</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A124" s="1">
+        <v>46082</v>
+      </c>
+      <c r="B124" s="2">
+        <v>4.4531908764296766</v>
+      </c>
+      <c r="C124" s="2">
+        <v>20.753485612577869</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>